<commit_message>
Update all models, add Graco (GGG)
</commit_message>
<xml_diff>
--- a/downloads/QLYS_Financial_Model.xlsx
+++ b/downloads/QLYS_Financial_Model.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/arijaymehta/Library/CloudStorage/GoogleDrive-asmehta4@gmail.com/My Drive/Stock Studies/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A86EFC6D-A622-E844-A4F6-1AE5EF9CEBD9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B59E863A-EBBD-C342-BBD6-BADCFA688CF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="38400" windowHeight="21000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="38400" windowHeight="21600" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cover Page" sheetId="16" r:id="rId1"/>
@@ -1337,9 +1337,6 @@
     <t>Buybacks compounding per-share value. ~2% annual share count reduction on top of organic growth</t>
   </si>
   <si>
-    <t>Platform is deep but narrow. Only provide vulnerability management and compliance. Bigger players offer end-to-end incl. endpoint, network and cloud</t>
-  </si>
-  <si>
     <t>CrowdStrike, Palo Alto, Zscaler competing for same enterprise wallet. Platform consolidation may favor larger vendors</t>
   </si>
   <si>
@@ -1978,11 +1975,6 @@
     <t>Price Line Y</t>
   </si>
   <si>
-    <t>Core Thesis — Why is QLYS at $80?
-The market is pricing in the liklihood that net retention will fall below 100% and cash flow erosion will ensue due to  platform consolidators (PANW, CRWD) bundling Vulnerability Managment (VM) into their suites and capping QLYS's pricing power on renewals. In addition, there may be terminal value doubt about QLYS existing as a standalone in 10 years.
-However, even in the bear case, margins protect the downside. At current profitability QLYS prints ~$225M/yr of true economic cash regardless of growth — a fair "no-growth" value is 10-12x FCF-ex-SBC = $90/sh. The question becomes whether that bear case actually plays out. If NDER stabilizes above 102% and S&amp;M discipline holds, the stock is meaningfully mispriced. If NDER keeps begins to slip and continues below 100%, the current price is fair.</t>
-  </si>
-  <si>
     <t>Growing buyback $ reflects growing FCF base, not just higher payout ratio.</t>
   </si>
   <si>
@@ -2005,6 +1997,15 @@
   </si>
   <si>
     <t>At $80.52, the market implies EV of ~$2,241M, or 3.4x EV/Revenue, 9.5x EV/EBITDA, and 7.4x EV/FCF. This is a meaningful discount to cyber peers (29x EV/EBITDA median).</t>
+  </si>
+  <si>
+    <t>Platform is deep but narrow. Only provide vulnerability management and compliance. Bigger players offer end-to-end incl. endpoint, network and cloud ****</t>
+  </si>
+  <si>
+    <t>Core Thesis — Why is QLYS at $80? The answer lies in terminal value assumptions.
+The market is pricing in the likelihood that net retention, though stable right now, falls below 100% in the future due to customer churn and price compression from platform consolidators (PANW, CRWD) bundling Vulnerability Management (VM) into their suites. Layered on top is terminal-value doubt about QLYS existing as a standalone in 10 years: does the VM product category exist as a standalone spend line in 2032 — yes or no?
+At current profitability QLYS prints ~$225M/yr of true economic cash regardless of growth. A fair "no-growth" value is 10–12x FCF-ex-SBC, or roughly $80–90/sh — meaning the stock is already trading at the low end of its no-growth floor. The question becomes which way it breaks from here. If NDER stabilizes above 102% and S&amp;M discipline holds, the stock is meaningfully mispriced to the upside. If NDER slips and sustains below 100%, the floor itself compresses (8–10x) as the market loses faith in standalone VM, and downside opens up.
+That being said, downside is cushioned by strategic value: at ~$225M of FCF, QLYS is an lucrative add-on for a platform player (PANW, CRWD, S) or a PE sponsor at a typical 15–18x FCF take-out, which brackets the current price. That optionality is why the stock is unlikely to trade materially below $80 absent a fundamental break in the cash flow profile.</t>
   </si>
 </sst>
 </file>
@@ -3846,7 +3847,7 @@
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
                   <c15:dlblFieldTable>
                     <c15:dlblFTEntry>
-                      <c15:txfldGUID>{F9F74D22-0233-6446-B449-E9D3A4B4FB60}</c15:txfldGUID>
+                      <c15:txfldGUID>{3DC51CA2-9AF5-E149-A311-597E7052AC48}</c15:txfldGUID>
                       <c15:f>'FootballField Data'!$F$6</c15:f>
                       <c15:dlblFieldTableCache>
                         <c:ptCount val="1"/>
@@ -3912,7 +3913,7 @@
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
                   <c15:dlblFieldTable>
                     <c15:dlblFTEntry>
-                      <c15:txfldGUID>{0D846F43-BD78-1945-BA5C-5B75038C357E}</c15:txfldGUID>
+                      <c15:txfldGUID>{FD3668AD-C83C-5D4A-A0B6-08D96FB391B5}</c15:txfldGUID>
                       <c15:f>'FootballField Data'!$F$7</c15:f>
                       <c15:dlblFieldTableCache>
                         <c:ptCount val="1"/>
@@ -3978,7 +3979,7 @@
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
                   <c15:dlblFieldTable>
                     <c15:dlblFTEntry>
-                      <c15:txfldGUID>{23D74FDC-CA71-6842-84AB-2867AA560016}</c15:txfldGUID>
+                      <c15:txfldGUID>{765CD4DE-0E4B-494F-9C83-2CEC2B2B1B09}</c15:txfldGUID>
                       <c15:f>'FootballField Data'!$F$8</c15:f>
                       <c15:dlblFieldTableCache>
                         <c:ptCount val="1"/>
@@ -4044,7 +4045,7 @@
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
                   <c15:dlblFieldTable>
                     <c15:dlblFTEntry>
-                      <c15:txfldGUID>{ADF9CE74-2039-E348-B2DA-8ECC15D1802C}</c15:txfldGUID>
+                      <c15:txfldGUID>{ABF1B530-3119-CA46-BF4C-3B01C76791BC}</c15:txfldGUID>
                       <c15:f>'FootballField Data'!$F$9</c15:f>
                       <c15:dlblFieldTableCache>
                         <c:ptCount val="1"/>
@@ -5328,17 +5329,17 @@
   <sheetData>
     <row r="2" spans="2:3" ht="42" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B2" s="386" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
     </row>
     <row r="3" spans="2:3" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B3" s="387" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
     </row>
     <row r="4" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B4" s="126" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
     </row>
     <row r="6" spans="2:3" s="21" customFormat="1" ht="16" customHeight="1" x14ac:dyDescent="0.2">
@@ -5393,7 +5394,7 @@
     </row>
     <row r="13" spans="2:3" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B13" s="162" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="C13" s="133"/>
     </row>
@@ -5408,7 +5409,7 @@
     </row>
     <row r="15" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B15" s="135" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="C15" s="136">
         <f>'DCF &amp; Sensitivity'!D53</f>
@@ -5417,7 +5418,7 @@
     </row>
     <row r="16" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B16" s="137" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="C16" s="138">
         <f>'DCF &amp; Sensitivity'!D54</f>
@@ -5430,7 +5431,7 @@
     </row>
     <row r="18" spans="2:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B18" s="162" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="C18" s="133"/>
     </row>
@@ -5463,7 +5464,7 @@
     </row>
     <row r="22" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B22" s="135" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="C22" s="139">
         <f>Assumptions!F11/100</f>
@@ -5472,7 +5473,7 @@
     </row>
     <row r="23" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B23" s="135" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="C23" s="139">
         <f>'Income Statement'!M28/100</f>
@@ -5481,7 +5482,7 @@
     </row>
     <row r="24" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B24" s="135" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="C24" s="141">
         <f>'DCF &amp; Sensitivity'!D48</f>
@@ -5490,7 +5491,7 @@
     </row>
     <row r="25" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B25" s="137" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="C25" s="142">
         <f>'DCF &amp; Sensitivity'!D51</f>
@@ -5509,85 +5510,85 @@
     </row>
     <row r="28" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B28" s="143" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="C28" s="4"/>
     </row>
     <row r="29" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B29" s="4" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="C29" s="4"/>
     </row>
     <row r="30" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B30" s="4" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="C30" s="4"/>
     </row>
     <row r="31" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B31" s="143" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="C31" s="4"/>
     </row>
     <row r="32" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B32" s="4" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="C32" s="4"/>
     </row>
     <row r="33" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B33" s="4" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="C33" s="4"/>
     </row>
     <row r="34" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B34" s="4" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="C34" s="4"/>
     </row>
     <row r="35" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B35" s="4" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="C35" s="4"/>
     </row>
     <row r="36" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B36" s="4" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="C36" s="4"/>
     </row>
     <row r="37" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B37" s="4" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="C37" s="4"/>
     </row>
     <row r="38" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B38" s="4" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="C38" s="4"/>
     </row>
     <row r="39" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B39" s="143" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="C39" s="4"/>
     </row>
     <row r="40" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B40" s="4" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="C40" s="4"/>
     </row>
     <row r="41" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B41" s="4" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="C41" s="4"/>
     </row>
@@ -5633,17 +5634,17 @@
     </row>
     <row r="6" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B6" s="278" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
     </row>
     <row r="7" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B7" s="3" t="s">
-        <v>536</v>
+        <v>534</v>
       </c>
     </row>
     <row r="8" spans="2:13" ht="41" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B8" s="395" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="C8" s="395"/>
       <c r="D8" s="395"/>
@@ -5656,7 +5657,7 @@
     </row>
     <row r="10" spans="2:13" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B10" s="271" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
       <c r="C10" s="96"/>
       <c r="D10" s="133"/>
@@ -5714,7 +5715,7 @@
     </row>
     <row r="13" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B13" s="8" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="C13" s="43" t="s">
         <v>5</v>
@@ -5886,40 +5887,40 @@
     </row>
     <row r="22" spans="2:15" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B22" s="271" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="C22" s="96" t="s">
         <v>13</v>
       </c>
       <c r="D22" s="287" t="s">
+        <v>443</v>
+      </c>
+      <c r="E22" s="287" t="s">
         <v>444</v>
       </c>
-      <c r="E22" s="287" t="s">
+      <c r="F22" s="287" t="s">
         <v>445</v>
       </c>
-      <c r="F22" s="287" t="s">
+      <c r="G22" s="287" t="s">
         <v>446</v>
       </c>
-      <c r="G22" s="287" t="s">
+      <c r="H22" s="287" t="s">
+        <v>439</v>
+      </c>
+      <c r="I22" s="288" t="s">
         <v>447</v>
       </c>
-      <c r="H22" s="287" t="s">
-        <v>440</v>
-      </c>
-      <c r="I22" s="288" t="s">
+      <c r="J22" s="288" t="s">
         <v>448</v>
       </c>
-      <c r="J22" s="288" t="s">
+      <c r="K22" s="288" t="s">
         <v>449</v>
       </c>
-      <c r="K22" s="288" t="s">
+      <c r="L22" s="288" t="s">
         <v>450</v>
       </c>
-      <c r="L22" s="288" t="s">
+      <c r="M22" s="288" t="s">
         <v>451</v>
-      </c>
-      <c r="M22" s="288" t="s">
-        <v>452</v>
       </c>
       <c r="O22" s="15" t="s">
         <v>95</v>
@@ -5958,7 +5959,7 @@
         <v>300.07834802779553</v>
       </c>
       <c r="O23" s="390" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
     </row>
     <row r="24" spans="2:15" x14ac:dyDescent="0.2">
@@ -6065,7 +6066,7 @@
       <c r="C28" s="96"/>
       <c r="D28" s="133"/>
       <c r="O28" s="396" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
     </row>
     <row r="29" spans="2:15" x14ac:dyDescent="0.2">
@@ -6194,12 +6195,12 @@
     <row r="40" spans="2:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="D40" s="88"/>
       <c r="O40" s="396" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
     </row>
     <row r="41" spans="2:15" ht="15" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B41" s="271" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="C41" s="96"/>
       <c r="D41" s="133"/>
@@ -6367,7 +6368,7 @@
         <v>80.52</v>
       </c>
       <c r="E55" s="4" t="s">
-        <v>483</v>
+        <v>482</v>
       </c>
       <c r="F55" s="88"/>
       <c r="O55" s="396"/>
@@ -6430,7 +6431,7 @@
     </row>
     <row r="64" spans="2:15" ht="15" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B64" s="272" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
       <c r="C64" s="273"/>
       <c r="D64" s="273"/>
@@ -6479,7 +6480,7 @@
         <v>12</v>
       </c>
       <c r="O66" s="390" t="s">
-        <v>482</v>
+        <v>481</v>
       </c>
     </row>
     <row r="67" spans="2:15" x14ac:dyDescent="0.2">
@@ -6679,7 +6680,7 @@
     </row>
     <row r="75" spans="2:15" ht="15" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B75" s="272" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
       <c r="C75" s="273"/>
       <c r="D75" s="273"/>
@@ -6951,7 +6952,7 @@
   <sheetData>
     <row r="2" spans="1:17" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B2" s="36" t="s">
-        <v>485</v>
+        <v>484</v>
       </c>
     </row>
     <row r="3" spans="1:17" ht="15" x14ac:dyDescent="0.2">
@@ -6969,7 +6970,7 @@
     </row>
     <row r="6" spans="1:17" ht="59" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B6" s="397" t="s">
-        <v>508</v>
+        <v>507</v>
       </c>
       <c r="C6" s="397"/>
       <c r="D6" s="397"/>
@@ -7013,13 +7014,13 @@
         <v>253</v>
       </c>
       <c r="D9" s="287" t="s">
+        <v>489</v>
+      </c>
+      <c r="E9" s="287" t="s">
         <v>490</v>
       </c>
-      <c r="E9" s="287" t="s">
-        <v>491</v>
-      </c>
       <c r="F9" s="287" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="G9" s="287" t="s">
         <v>255</v>
@@ -7028,19 +7029,19 @@
         <v>256</v>
       </c>
       <c r="I9" s="287" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
       <c r="J9" s="287" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
       <c r="K9" s="287" t="s">
+        <v>491</v>
+      </c>
+      <c r="L9" s="287" t="s">
         <v>492</v>
       </c>
-      <c r="L9" s="287" t="s">
+      <c r="M9" s="287" t="s">
         <v>493</v>
-      </c>
-      <c r="M9" s="287" t="s">
-        <v>494</v>
       </c>
       <c r="N9" s="287" t="s">
         <v>258</v>
@@ -7049,10 +7050,10 @@
         <v>259</v>
       </c>
       <c r="P9" s="287" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="Q9" s="314" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
     </row>
     <row r="10" spans="1:17" x14ac:dyDescent="0.2">
@@ -7154,7 +7155,7 @@
     <row r="13" spans="1:17" ht="15" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A13" s="143"/>
       <c r="B13" s="272" t="s">
-        <v>484</v>
+        <v>483</v>
       </c>
       <c r="C13" s="273"/>
       <c r="D13" s="273"/>
@@ -7504,7 +7505,7 @@
         <v>-125</v>
       </c>
       <c r="Q19" s="336" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
     </row>
     <row r="20" spans="2:17" x14ac:dyDescent="0.2">
@@ -7615,7 +7616,7 @@
         <v>-85</v>
       </c>
       <c r="Q21" s="336" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
     </row>
     <row r="22" spans="2:17" x14ac:dyDescent="0.2">
@@ -7693,7 +7694,7 @@
     </row>
     <row r="24" spans="2:17" ht="15" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B24" s="272" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="C24" s="273"/>
       <c r="D24" s="273"/>
@@ -7713,7 +7714,7 @@
     </row>
     <row r="25" spans="2:17" x14ac:dyDescent="0.2">
       <c r="B25" s="337" t="s">
-        <v>505</v>
+        <v>504</v>
       </c>
       <c r="C25" s="337"/>
       <c r="D25" s="330">
@@ -7775,7 +7776,7 @@
     </row>
     <row r="26" spans="2:17" x14ac:dyDescent="0.2">
       <c r="B26" s="119" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
       <c r="C26" s="119"/>
       <c r="D26" s="330">
@@ -7869,7 +7870,7 @@
     </row>
     <row r="29" spans="2:17" ht="15" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B29" s="272" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="C29" s="273"/>
       <c r="D29" s="273"/>
@@ -7883,26 +7884,26 @@
     </row>
     <row r="30" spans="2:17" x14ac:dyDescent="0.2">
       <c r="B30" s="321" t="s">
-        <v>486</v>
+        <v>485</v>
       </c>
       <c r="C30" s="322"/>
       <c r="D30" s="322" t="s">
+        <v>496</v>
+      </c>
+      <c r="E30" s="322" t="s">
         <v>497</v>
       </c>
-      <c r="E30" s="322" t="s">
+      <c r="F30" s="322" t="s">
+        <v>486</v>
+      </c>
+      <c r="G30" s="322" t="s">
         <v>498</v>
       </c>
-      <c r="F30" s="322" t="s">
+      <c r="H30" s="322" t="s">
+        <v>499</v>
+      </c>
+      <c r="I30" s="322" t="s">
         <v>487</v>
-      </c>
-      <c r="G30" s="322" t="s">
-        <v>499</v>
-      </c>
-      <c r="H30" s="322" t="s">
-        <v>500</v>
-      </c>
-      <c r="I30" s="322" t="s">
-        <v>488</v>
       </c>
       <c r="K30" s="120"/>
       <c r="O30" s="21"/>
@@ -7939,7 +7940,7 @@
     </row>
     <row r="32" spans="2:17" x14ac:dyDescent="0.2">
       <c r="B32" s="311" t="s">
-        <v>501</v>
+        <v>500</v>
       </c>
       <c r="C32" s="29"/>
       <c r="D32" s="299">
@@ -7997,7 +7998,7 @@
     </row>
     <row r="34" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B34" s="311" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="C34" s="29"/>
       <c r="D34" s="299">
@@ -8035,7 +8036,7 @@
     </row>
     <row r="36" spans="2:9" ht="15" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B36" s="272" t="s">
-        <v>495</v>
+        <v>494</v>
       </c>
       <c r="C36" s="273"/>
       <c r="D36" s="273"/>
@@ -8047,7 +8048,7 @@
     </row>
     <row r="37" spans="2:9" ht="14" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B37" s="398" t="s">
-        <v>507</v>
+        <v>506</v>
       </c>
       <c r="C37" s="398"/>
       <c r="D37" s="398"/>
@@ -8160,7 +8161,7 @@
   <sheetData>
     <row r="18" spans="2:2" ht="24" x14ac:dyDescent="0.3">
       <c r="B18" s="128" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
     </row>
   </sheetData>
@@ -8298,10 +8299,10 @@
     </row>
     <row r="21" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B21" s="68" t="s">
+        <v>428</v>
+      </c>
+      <c r="C21" s="68" t="s">
         <v>429</v>
-      </c>
-      <c r="C21" s="68" t="s">
-        <v>430</v>
       </c>
     </row>
     <row r="22" spans="2:3" x14ac:dyDescent="0.2">
@@ -8356,12 +8357,12 @@
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A1" s="4" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B2" s="400" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="C2" s="400"/>
       <c r="D2" s="400"/>
@@ -8369,25 +8370,25 @@
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B3" s="127" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B4" s="127" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B6" s="346" t="s">
+        <v>363</v>
+      </c>
+      <c r="C6" s="127" t="s">
         <v>364</v>
-      </c>
-      <c r="C6" s="127" t="s">
-        <v>365</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B8" s="347" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="C8" s="347" t="s">
         <v>13</v>
@@ -8413,7 +8414,7 @@
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B9" s="348" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="C9" s="6" t="s">
         <v>25</v>
@@ -8445,7 +8446,7 @@
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B10" s="350" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="C10" s="6" t="s">
         <v>3</v>
@@ -8505,7 +8506,7 @@
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B12" s="6" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="C12" s="6" t="s">
         <v>3</v>
@@ -8535,7 +8536,7 @@
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B13" s="6" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="C13" s="6" t="s">
         <v>3</v>
@@ -8565,7 +8566,7 @@
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B14" s="6" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="C14" s="6" t="s">
         <v>3</v>
@@ -8625,7 +8626,7 @@
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B16" s="348" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="C16" s="6" t="s">
         <v>25</v>
@@ -8655,7 +8656,7 @@
     </row>
     <row r="17" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B17" s="6" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="C17" s="6" t="s">
         <v>25</v>
@@ -8685,7 +8686,7 @@
     </row>
     <row r="18" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B18" s="348" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="C18" s="6" t="s">
         <v>25</v>
@@ -8715,7 +8716,7 @@
     </row>
     <row r="19" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B19" s="348" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="C19" s="6" t="s">
         <v>25</v>
@@ -8745,7 +8746,7 @@
     </row>
     <row r="20" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B20" s="348" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="C20" s="6" t="s">
         <v>25</v>
@@ -8775,7 +8776,7 @@
     </row>
     <row r="21" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B21" s="348" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="C21" s="6" t="s">
         <v>25</v>
@@ -8805,7 +8806,7 @@
     </row>
     <row r="22" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B22" s="355" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="C22" s="6" t="s">
         <v>25</v>
@@ -8835,7 +8836,7 @@
     </row>
     <row r="23" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B23" s="356" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="C23" s="4" t="s">
         <v>25</v>
@@ -8918,7 +8919,7 @@
     </row>
     <row r="27" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B27" s="348" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="C27" s="6" t="s">
         <v>25</v>
@@ -8965,7 +8966,7 @@
     </row>
     <row r="30" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B30" s="348" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="C30" s="6" t="s">
         <v>25</v>
@@ -8977,7 +8978,7 @@
     </row>
     <row r="31" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B31" s="348" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="C31" s="6" t="s">
         <v>25</v>
@@ -8989,7 +8990,7 @@
     </row>
     <row r="32" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B32" s="348" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="C32" s="6" t="s">
         <v>25</v>
@@ -9001,7 +9002,7 @@
     </row>
     <row r="33" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B33" s="348" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="C33" s="6" t="s">
         <v>25</v>
@@ -9037,7 +9038,7 @@
     </row>
     <row r="36" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B36" s="348" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="C36" s="6" t="s">
         <v>25</v>
@@ -9073,7 +9074,7 @@
     </row>
     <row r="39" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B39" s="359" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="C39" s="6" t="s">
         <v>49</v>
@@ -9085,7 +9086,7 @@
     </row>
     <row r="40" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B40" s="359" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="C40" s="6" t="s">
         <v>49</v>
@@ -9097,15 +9098,15 @@
     </row>
     <row r="42" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B42" s="361" t="s">
+        <v>384</v>
+      </c>
+      <c r="C42" s="127" t="s">
         <v>385</v>
-      </c>
-      <c r="C42" s="127" t="s">
-        <v>386</v>
       </c>
     </row>
     <row r="44" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B44" s="347" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="C44" s="347" t="s">
         <v>13</v>
@@ -9131,7 +9132,7 @@
     </row>
     <row r="45" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B45" s="348" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="C45" s="6" t="s">
         <v>25</v>
@@ -9163,7 +9164,7 @@
     </row>
     <row r="46" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B46" s="350" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="C46" s="6" t="s">
         <v>3</v>
@@ -9223,7 +9224,7 @@
     </row>
     <row r="48" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B48" s="6" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="C48" s="6" t="s">
         <v>3</v>
@@ -9253,7 +9254,7 @@
     </row>
     <row r="49" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B49" s="6" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="C49" s="6" t="s">
         <v>3</v>
@@ -9283,7 +9284,7 @@
     </row>
     <row r="50" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B50" s="6" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="C50" s="6" t="s">
         <v>3</v>
@@ -9343,7 +9344,7 @@
     </row>
     <row r="52" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B52" s="348" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="C52" s="6" t="s">
         <v>25</v>
@@ -9373,7 +9374,7 @@
     </row>
     <row r="53" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B53" s="6" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="C53" s="6" t="s">
         <v>25</v>
@@ -9403,7 +9404,7 @@
     </row>
     <row r="54" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B54" s="348" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="C54" s="6" t="s">
         <v>25</v>
@@ -9433,7 +9434,7 @@
     </row>
     <row r="55" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B55" s="348" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="C55" s="6" t="s">
         <v>25</v>
@@ -9463,7 +9464,7 @@
     </row>
     <row r="56" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B56" s="348" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="C56" s="6" t="s">
         <v>25</v>
@@ -9493,7 +9494,7 @@
     </row>
     <row r="57" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B57" s="348" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="C57" s="6" t="s">
         <v>25</v>
@@ -9523,7 +9524,7 @@
     </row>
     <row r="58" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B58" s="355" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="C58" s="6" t="s">
         <v>25</v>
@@ -9553,7 +9554,7 @@
     </row>
     <row r="59" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B59" s="362" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="C59" s="6" t="s">
         <v>25</v>
@@ -9638,7 +9639,7 @@
     </row>
     <row r="63" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B63" s="348" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="C63" s="6" t="s">
         <v>25</v>
@@ -9685,7 +9686,7 @@
     </row>
     <row r="66" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B66" s="348" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="C66" s="6" t="s">
         <v>25</v>
@@ -9697,7 +9698,7 @@
     </row>
     <row r="67" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B67" s="348" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="C67" s="6" t="s">
         <v>25</v>
@@ -9709,7 +9710,7 @@
     </row>
     <row r="68" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B68" s="348" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="C68" s="6" t="s">
         <v>25</v>
@@ -9721,7 +9722,7 @@
     </row>
     <row r="69" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B69" s="348" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="C69" s="6" t="s">
         <v>25</v>
@@ -9757,7 +9758,7 @@
     </row>
     <row r="72" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B72" s="348" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="C72" s="6" t="s">
         <v>25</v>
@@ -9793,7 +9794,7 @@
     </row>
     <row r="75" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B75" s="359" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="C75" s="6" t="s">
         <v>49</v>
@@ -9805,7 +9806,7 @@
     </row>
     <row r="76" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B76" s="289" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="C76" s="4" t="s">
         <v>49</v>
@@ -9817,15 +9818,15 @@
     </row>
     <row r="78" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B78" s="365" t="s">
+        <v>386</v>
+      </c>
+      <c r="C78" s="127" t="s">
         <v>387</v>
-      </c>
-      <c r="C78" s="127" t="s">
-        <v>388</v>
       </c>
     </row>
     <row r="80" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B80" s="347" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="C80" s="347" t="s">
         <v>13</v>
@@ -9851,7 +9852,7 @@
     </row>
     <row r="81" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B81" s="348" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="C81" s="6" t="s">
         <v>25</v>
@@ -9883,7 +9884,7 @@
     </row>
     <row r="82" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B82" s="350" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="C82" s="6" t="s">
         <v>3</v>
@@ -9943,7 +9944,7 @@
     </row>
     <row r="84" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B84" s="6" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="C84" s="6" t="s">
         <v>3</v>
@@ -9973,7 +9974,7 @@
     </row>
     <row r="85" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B85" s="6" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="C85" s="6" t="s">
         <v>3</v>
@@ -10003,7 +10004,7 @@
     </row>
     <row r="86" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B86" s="6" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="C86" s="6" t="s">
         <v>3</v>
@@ -10063,7 +10064,7 @@
     </row>
     <row r="88" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B88" s="348" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="C88" s="6" t="s">
         <v>25</v>
@@ -10093,7 +10094,7 @@
     </row>
     <row r="89" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B89" s="6" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="C89" s="6" t="s">
         <v>25</v>
@@ -10123,7 +10124,7 @@
     </row>
     <row r="90" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B90" s="348" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="C90" s="6" t="s">
         <v>25</v>
@@ -10153,7 +10154,7 @@
     </row>
     <row r="91" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B91" s="348" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="C91" s="6" t="s">
         <v>25</v>
@@ -10183,7 +10184,7 @@
     </row>
     <row r="92" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B92" s="348" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="C92" s="6" t="s">
         <v>25</v>
@@ -10213,7 +10214,7 @@
     </row>
     <row r="93" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B93" s="348" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="C93" s="6" t="s">
         <v>25</v>
@@ -10243,7 +10244,7 @@
     </row>
     <row r="94" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B94" s="355" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="C94" s="6" t="s">
         <v>25</v>
@@ -10273,7 +10274,7 @@
     </row>
     <row r="95" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B95" s="362" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="C95" s="6" t="s">
         <v>25</v>
@@ -10358,7 +10359,7 @@
     </row>
     <row r="99" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B99" s="348" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="C99" s="6" t="s">
         <v>25</v>
@@ -10405,7 +10406,7 @@
     </row>
     <row r="102" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B102" s="348" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="C102" s="6" t="s">
         <v>25</v>
@@ -10417,7 +10418,7 @@
     </row>
     <row r="103" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B103" s="348" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="C103" s="6" t="s">
         <v>25</v>
@@ -10429,7 +10430,7 @@
     </row>
     <row r="104" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B104" s="348" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="C104" s="6" t="s">
         <v>25</v>
@@ -10441,7 +10442,7 @@
     </row>
     <row r="105" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B105" s="348" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="C105" s="6" t="s">
         <v>25</v>
@@ -10477,7 +10478,7 @@
     </row>
     <row r="108" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B108" s="348" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="C108" s="6" t="s">
         <v>25</v>
@@ -10513,7 +10514,7 @@
     </row>
     <row r="111" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B111" s="359" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="C111" s="6" t="s">
         <v>49</v>
@@ -10525,7 +10526,7 @@
     </row>
     <row r="112" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B112" s="359" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="C112" s="6" t="s">
         <v>49</v>
@@ -10556,43 +10557,43 @@
   <sheetData>
     <row r="1" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A1" s="165" t="s">
-        <v>512</v>
+        <v>511</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A3" s="381" t="s">
-        <v>513</v>
+        <v>512</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A5" s="382" t="s">
-        <v>486</v>
+        <v>485</v>
       </c>
       <c r="B5" s="382" t="s">
+        <v>513</v>
+      </c>
+      <c r="C5" s="382" t="s">
         <v>514</v>
       </c>
-      <c r="C5" s="382" t="s">
+      <c r="D5" s="382" t="s">
         <v>515</v>
       </c>
-      <c r="D5" s="382" t="s">
+      <c r="E5" s="382" t="s">
         <v>516</v>
       </c>
-      <c r="E5" s="382" t="s">
-        <v>517</v>
-      </c>
       <c r="F5" s="382" t="s">
+        <v>525</v>
+      </c>
+      <c r="H5" s="382" t="s">
         <v>526</v>
       </c>
-      <c r="H5" s="382" t="s">
+      <c r="I5" s="382" t="s">
         <v>527</v>
-      </c>
-      <c r="I5" s="382" t="s">
-        <v>528</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
       <c r="B6" s="383">
         <f>'Scenario Summary'!D8</f>
@@ -10607,7 +10608,7 @@
         <v>179.13503447024598</v>
       </c>
       <c r="E6" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="F6" t="str">
         <f>"$"&amp;TEXT(B6,"#,##0")&amp;" – $"&amp;TEXT(D6,"#,##0")</f>
@@ -10623,7 +10624,7 @@
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
       <c r="B7" s="383">
         <f>'Scenario Summary'!D9</f>
@@ -10638,7 +10639,7 @@
         <v>261.01640854386812</v>
       </c>
       <c r="E7" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="F7" t="str">
         <f>"$"&amp;TEXT(B7,"#,##0")&amp;" – $"&amp;TEXT(D7,"#,##0")</f>
@@ -10654,7 +10655,7 @@
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
       <c r="B8" s="383">
         <f>(PERCENTILE(Comps!N14:N22,0.25)*'Income Statement'!I47-'DCF &amp; Sensitivity'!D48)/Assumptions!I64</f>
@@ -10669,7 +10670,7 @@
         <v>109.27935933354455</v>
       </c>
       <c r="E8" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
       <c r="F8" t="str">
         <f>"$"&amp;TEXT(B8,"#,##0")&amp;" – $"&amp;TEXT(D8,"#,##0")</f>
@@ -10678,7 +10679,7 @@
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="B9" s="383">
         <v>74.510000000000005</v>
@@ -10691,7 +10692,7 @@
         <v>155.47</v>
       </c>
       <c r="E9" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="F9" t="str">
         <f>"$"&amp;TEXT(B9,"#,##0")&amp;" – $"&amp;TEXT(D9,"#,##0")</f>
@@ -10700,7 +10701,7 @@
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A11" s="125" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="B11" s="383">
         <f>'DCF &amp; Sensitivity'!D55</f>
@@ -10729,25 +10730,25 @@
   <sheetData>
     <row r="2" spans="2:7" ht="26" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B2" s="165" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="C2" s="165"/>
     </row>
     <row r="3" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B3" s="5" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="C3" s="5"/>
     </row>
     <row r="4" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B4" s="166" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="C4" s="166"/>
     </row>
     <row r="5" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B5" s="167" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
       <c r="C5" s="167"/>
       <c r="D5" s="4"/>
@@ -10765,7 +10766,7 @@
     </row>
     <row r="7" spans="2:7" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B7" s="172" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="C7" s="172" t="s">
         <v>13</v>
@@ -10780,12 +10781,12 @@
         <v>68</v>
       </c>
       <c r="G7" s="376" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
     </row>
     <row r="8" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B8" s="144" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="C8" s="144" t="s">
         <v>49</v>
@@ -10809,7 +10810,7 @@
     </row>
     <row r="9" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B9" s="6" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="C9" s="6" t="s">
         <v>49</v>
@@ -10833,7 +10834,7 @@
     </row>
     <row r="10" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B10" s="6" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="C10" s="6" t="s">
         <v>49</v>
@@ -10875,12 +10876,12 @@
         <v>80.52</v>
       </c>
       <c r="G11" s="370" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
     </row>
     <row r="12" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B12" s="155" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="C12" s="6" t="s">
         <v>3</v>
@@ -10912,7 +10913,7 @@
     </row>
     <row r="14" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B14" s="168" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
       <c r="C14" s="168" t="s">
         <v>13</v>
@@ -10927,7 +10928,7 @@
         <v>68</v>
       </c>
       <c r="G14" s="375" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
     </row>
     <row r="15" spans="2:7" x14ac:dyDescent="0.2">
@@ -10980,7 +10981,7 @@
     </row>
     <row r="17" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B17" s="6" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="C17" s="6" t="s">
         <v>90</v>
@@ -11094,7 +11095,7 @@
         <v>3.5</v>
       </c>
       <c r="G21" s="159" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
     </row>
     <row r="22" spans="2:7" x14ac:dyDescent="0.2">
@@ -11117,12 +11118,12 @@
         <v>25</v>
       </c>
       <c r="G22" s="371" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
     </row>
     <row r="23" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B23" s="155" t="s">
-        <v>509</v>
+        <v>508</v>
       </c>
       <c r="C23" s="155" t="s">
         <v>3</v>
@@ -11154,7 +11155,7 @@
     </row>
     <row r="25" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B25" s="168" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="C25" s="168" t="s">
         <v>13</v>
@@ -11193,7 +11194,7 @@
     </row>
     <row r="27" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B27" s="155" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="C27" s="155" t="s">
         <v>3</v>
@@ -11235,7 +11236,7 @@
     </row>
     <row r="29" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B29" s="6" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="C29" s="6" t="s">
         <v>25</v>
@@ -11256,7 +11257,7 @@
     </row>
     <row r="30" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B30" s="6" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="C30" s="6" t="s">
         <v>25</v>
@@ -11277,7 +11278,7 @@
     </row>
     <row r="31" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B31" s="6" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="C31" s="6" t="s">
         <v>25</v>
@@ -11298,7 +11299,7 @@
     </row>
     <row r="32" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B32" s="6" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
       <c r="C32" s="6" t="s">
         <v>25</v>
@@ -11327,7 +11328,7 @@
     </row>
     <row r="34" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B34" s="162" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
       <c r="C34" s="162"/>
       <c r="D34" s="162"/>
@@ -11337,7 +11338,7 @@
     </row>
     <row r="35" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B35" s="389" t="s">
-        <v>529</v>
+        <v>536</v>
       </c>
       <c r="C35" s="390"/>
       <c r="D35" s="390"/>
@@ -11393,7 +11394,7 @@
       <c r="F41" s="390"/>
       <c r="G41" s="390"/>
     </row>
-    <row r="42" spans="2:7" ht="40" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="42" spans="2:7" ht="84" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B42" s="390"/>
       <c r="C42" s="390"/>
       <c r="D42" s="390"/>
@@ -11519,7 +11520,7 @@
         <v>6</v>
       </c>
       <c r="C11" s="65" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
     </row>
     <row r="12" spans="2:9" x14ac:dyDescent="0.2">
@@ -11575,7 +11576,7 @@
         <v>3</v>
       </c>
       <c r="C17" s="68" t="s">
-        <v>324</v>
+        <v>535</v>
       </c>
       <c r="D17" s="43"/>
       <c r="E17" s="43"/>
@@ -11589,7 +11590,7 @@
         <v>4</v>
       </c>
       <c r="C18" s="68" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="D18" s="43"/>
       <c r="E18" s="43"/>
@@ -11657,7 +11658,7 @@
         <v>4</v>
       </c>
       <c r="C24" s="68" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="D24" s="43"/>
       <c r="E24" s="43"/>
@@ -11683,7 +11684,7 @@
         <v>1</v>
       </c>
       <c r="C27" s="68" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="D27" s="43"/>
       <c r="E27" s="43"/>
@@ -11697,7 +11698,7 @@
         <v>2</v>
       </c>
       <c r="C28" s="68" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="D28" s="43"/>
       <c r="E28" s="43"/>
@@ -11711,7 +11712,7 @@
         <v>3</v>
       </c>
       <c r="C29" s="68" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="D29" s="43"/>
       <c r="E29" s="43"/>
@@ -11725,7 +11726,7 @@
         <v>4</v>
       </c>
       <c r="C30" s="68" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="D30" s="43"/>
       <c r="E30" s="43"/>
@@ -11752,7 +11753,7 @@
   <sheetData>
     <row r="18" spans="2:2" ht="24" x14ac:dyDescent="0.3">
       <c r="B18" s="128" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
     </row>
   </sheetData>
@@ -11805,7 +11806,7 @@
     </row>
     <row r="8" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B8" s="176" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="C8" s="98"/>
       <c r="D8" s="98"/>
@@ -11918,7 +11919,7 @@
     </row>
     <row r="14" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B14" s="177" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="C14" s="234"/>
       <c r="D14" s="100"/>
@@ -11998,7 +11999,7 @@
     </row>
     <row r="18" spans="1:15" x14ac:dyDescent="0.2">
       <c r="B18" s="177" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="C18" s="234"/>
       <c r="D18" s="100"/>
@@ -12066,7 +12067,7 @@
     </row>
     <row r="22" spans="1:15" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B22" s="212" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="C22" s="238" t="s">
         <v>3</v>
@@ -12113,34 +12114,34 @@
         <v>13</v>
       </c>
       <c r="D25" s="180" t="s">
+        <v>443</v>
+      </c>
+      <c r="E25" s="180" t="s">
         <v>444</v>
       </c>
-      <c r="E25" s="180" t="s">
+      <c r="F25" s="180" t="s">
         <v>445</v>
       </c>
-      <c r="F25" s="180" t="s">
+      <c r="G25" s="180" t="s">
         <v>446</v>
       </c>
-      <c r="G25" s="180" t="s">
+      <c r="H25" s="180" t="s">
+        <v>439</v>
+      </c>
+      <c r="I25" s="181" t="s">
         <v>447</v>
       </c>
-      <c r="H25" s="180" t="s">
-        <v>440</v>
-      </c>
-      <c r="I25" s="181" t="s">
+      <c r="J25" s="181" t="s">
         <v>448</v>
       </c>
-      <c r="J25" s="181" t="s">
+      <c r="K25" s="181" t="s">
         <v>449</v>
       </c>
-      <c r="K25" s="181" t="s">
+      <c r="L25" s="181" t="s">
         <v>450</v>
       </c>
-      <c r="L25" s="181" t="s">
+      <c r="M25" s="181" t="s">
         <v>451</v>
-      </c>
-      <c r="M25" s="181" t="s">
-        <v>452</v>
       </c>
       <c r="O25" s="15" t="s">
         <v>95</v>
@@ -12716,7 +12717,7 @@
     </row>
     <row r="42" spans="2:15" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B42" s="217" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="C42" s="218"/>
       <c r="D42" s="219"/>
@@ -12880,7 +12881,7 @@
         <v>21.5</v>
       </c>
       <c r="O45" s="16" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
     </row>
     <row r="46" spans="2:15" x14ac:dyDescent="0.2">
@@ -13137,7 +13138,7 @@
         <v>93</v>
       </c>
       <c r="O52" s="16" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
     </row>
     <row r="53" spans="1:15" x14ac:dyDescent="0.2">
@@ -13323,7 +13324,7 @@
     </row>
     <row r="57" spans="1:15" x14ac:dyDescent="0.2">
       <c r="B57" s="14" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="C57" s="227" t="s">
         <v>3</v>
@@ -13391,15 +13392,15 @@
       <c r="L59" s="219"/>
       <c r="M59" s="219"/>
       <c r="O59" s="14" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
     </row>
     <row r="60" spans="1:15" x14ac:dyDescent="0.2">
       <c r="B60" s="185" t="s">
+        <v>452</v>
+      </c>
+      <c r="C60" s="228" t="s">
         <v>453</v>
-      </c>
-      <c r="C60" s="228" t="s">
-        <v>454</v>
       </c>
       <c r="D60" s="186">
         <v>138</v>
@@ -13437,13 +13438,13 @@
         <v>80.52</v>
       </c>
       <c r="O60" s="16" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
     </row>
     <row r="61" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A61" s="20"/>
       <c r="B61" s="189" t="s">
-        <v>455</v>
+        <v>454</v>
       </c>
       <c r="C61" s="229" t="s">
         <v>3</v>
@@ -13489,13 +13490,13 @@
         <v>80</v>
       </c>
       <c r="O61" s="16" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
     </row>
     <row r="62" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A62" s="56"/>
       <c r="B62" s="189" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
       <c r="C62" s="229" t="s">
         <v>25</v>
@@ -13541,7 +13542,7 @@
         <v>317.91026951269441</v>
       </c>
       <c r="O62" s="16" t="s">
-        <v>530</v>
+        <v>528</v>
       </c>
     </row>
     <row r="63" spans="1:15" x14ac:dyDescent="0.2">
@@ -13594,7 +13595,7 @@
     <row r="64" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A64" s="56"/>
       <c r="B64" s="189" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="C64" s="229" t="s">
         <v>47</v>
@@ -13636,13 +13637,13 @@
       </c>
       <c r="N64" s="56"/>
       <c r="O64" s="14" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
     </row>
     <row r="65" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A65" s="56"/>
       <c r="B65" s="196" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="C65" s="230" t="s">
         <v>3</v>
@@ -13689,7 +13690,7 @@
       </c>
       <c r="N65" s="56"/>
       <c r="O65" s="16" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
     </row>
     <row r="66" spans="1:15" x14ac:dyDescent="0.2">
@@ -13750,7 +13751,7 @@
     <row r="70" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A70" s="56"/>
       <c r="B70" s="29" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="C70" s="222" t="s">
         <v>5</v>
@@ -13764,7 +13765,7 @@
     <row r="71" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A71" s="56"/>
       <c r="B71" s="29" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="C71" s="222"/>
       <c r="D71" s="150">
@@ -13942,7 +13943,7 @@
     </row>
     <row r="6" spans="2:13" ht="14" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B6" s="391" t="s">
-        <v>531</v>
+        <v>529</v>
       </c>
       <c r="C6" s="391"/>
       <c r="D6" s="391"/>
@@ -14223,7 +14224,7 @@
         <v>101</v>
       </c>
       <c r="O21" s="16" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
     </row>
     <row r="22" spans="2:15" x14ac:dyDescent="0.2">
@@ -14317,7 +14318,7 @@
         <v>95.324196999531608</v>
       </c>
       <c r="O23" s="14" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
     </row>
     <row r="25" spans="2:15" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
@@ -14721,7 +14722,7 @@
     </row>
     <row r="37" spans="2:15" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B37" s="242" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="C37" s="242"/>
       <c r="D37" s="242"/>
@@ -14737,7 +14738,7 @@
     </row>
     <row r="38" spans="2:15" x14ac:dyDescent="0.2">
       <c r="B38" s="23" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="C38" s="23" t="s">
         <v>27</v>
@@ -14782,7 +14783,7 @@
         <v>10000</v>
       </c>
       <c r="O38" s="16" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
     </row>
     <row r="39" spans="2:15" x14ac:dyDescent="0.2">
@@ -14830,7 +14831,7 @@
         <v>1300</v>
       </c>
       <c r="O39" s="14" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
     </row>
     <row r="40" spans="2:15" x14ac:dyDescent="0.2">
@@ -14924,12 +14925,12 @@
         <v>13</v>
       </c>
       <c r="O41" s="14" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
     </row>
     <row r="42" spans="2:15" x14ac:dyDescent="0.2">
       <c r="B42" s="29" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="C42" s="29" t="s">
         <v>27</v>
@@ -15108,34 +15109,34 @@
         <v>13</v>
       </c>
       <c r="D6" s="240" t="s">
+        <v>443</v>
+      </c>
+      <c r="E6" s="240" t="s">
         <v>444</v>
       </c>
-      <c r="E6" s="240" t="s">
+      <c r="F6" s="240" t="s">
         <v>445</v>
       </c>
-      <c r="F6" s="240" t="s">
+      <c r="G6" s="240" t="s">
         <v>446</v>
       </c>
-      <c r="G6" s="240" t="s">
+      <c r="H6" s="240" t="s">
+        <v>439</v>
+      </c>
+      <c r="I6" s="241" t="s">
         <v>447</v>
       </c>
-      <c r="H6" s="240" t="s">
-        <v>440</v>
-      </c>
-      <c r="I6" s="241" t="s">
+      <c r="J6" s="241" t="s">
         <v>448</v>
       </c>
-      <c r="J6" s="241" t="s">
+      <c r="K6" s="241" t="s">
         <v>449</v>
       </c>
-      <c r="K6" s="241" t="s">
+      <c r="L6" s="241" t="s">
         <v>450</v>
       </c>
-      <c r="L6" s="241" t="s">
+      <c r="M6" s="241" t="s">
         <v>451</v>
-      </c>
-      <c r="M6" s="241" t="s">
-        <v>452</v>
       </c>
       <c r="O6" s="15" t="s">
         <v>95</v>
@@ -15143,7 +15144,7 @@
     </row>
     <row r="8" spans="2:15" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B8" s="178" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="C8" s="243"/>
       <c r="D8" s="244"/>
@@ -15205,7 +15206,7 @@
         <v>973.09488863072499</v>
       </c>
       <c r="O9" s="390" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
     </row>
     <row r="10" spans="2:15" s="14" customFormat="1" x14ac:dyDescent="0.2">
@@ -15313,7 +15314,7 @@
         <v>150.82970773776239</v>
       </c>
       <c r="O13" s="392" t="s">
-        <v>533</v>
+        <v>531</v>
       </c>
     </row>
     <row r="14" spans="2:15" x14ac:dyDescent="0.2">
@@ -15419,7 +15420,7 @@
     </row>
     <row r="17" spans="2:15" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B17" s="178" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
       <c r="C17" s="243"/>
       <c r="D17" s="244"/>
@@ -15477,7 +15478,7 @@
         <v>170.29160551037685</v>
       </c>
       <c r="O18" s="392" t="s">
-        <v>532</v>
+        <v>530</v>
       </c>
     </row>
     <row r="19" spans="2:15" x14ac:dyDescent="0.2">
@@ -15864,7 +15865,7 @@
         <v>345.4486854639074</v>
       </c>
       <c r="O27" s="394" t="s">
-        <v>534</v>
+        <v>532</v>
       </c>
     </row>
     <row r="28" spans="2:15" x14ac:dyDescent="0.2">
@@ -15921,7 +15922,7 @@
     </row>
     <row r="30" spans="2:15" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B30" s="178" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
       <c r="C30" s="243"/>
       <c r="D30" s="244"/>
@@ -15974,7 +15975,7 @@
         <v>17.5</v>
       </c>
       <c r="O31" s="392" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
     </row>
     <row r="32" spans="2:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -16266,7 +16267,7 @@
     </row>
     <row r="39" spans="2:15" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B39" s="178" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="C39" s="243"/>
       <c r="D39" s="244"/>
@@ -16329,7 +16330,7 @@
         <v>26.453210151175963</v>
       </c>
       <c r="O40" s="392" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
     </row>
     <row r="41" spans="2:15" x14ac:dyDescent="0.2">
@@ -16432,7 +16433,7 @@
     </row>
     <row r="44" spans="2:15" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B44" s="178" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="C44" s="243"/>
       <c r="D44" s="244"/>
@@ -16490,7 +16491,7 @@
         <v>10.704043774937976</v>
       </c>
       <c r="O45" s="392" t="s">
-        <v>535</v>
+        <v>533</v>
       </c>
     </row>
     <row r="46" spans="2:15" x14ac:dyDescent="0.2">
@@ -16686,7 +16687,7 @@
     </row>
     <row r="50" spans="2:15" x14ac:dyDescent="0.2">
       <c r="B50" s="21" t="s">
-        <v>474</v>
+        <v>473</v>
       </c>
       <c r="C50" s="29" t="s">
         <v>25</v>
@@ -16735,7 +16736,7 @@
     </row>
     <row r="51" spans="2:15" x14ac:dyDescent="0.2">
       <c r="B51" s="25" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="C51" s="25" t="s">
         <v>3</v>
@@ -16835,34 +16836,34 @@
         <v>13</v>
       </c>
       <c r="D6" s="240" t="s">
+        <v>443</v>
+      </c>
+      <c r="E6" s="240" t="s">
         <v>444</v>
       </c>
-      <c r="E6" s="240" t="s">
+      <c r="F6" s="240" t="s">
         <v>445</v>
       </c>
-      <c r="F6" s="240" t="s">
+      <c r="G6" s="240" t="s">
         <v>446</v>
       </c>
-      <c r="G6" s="240" t="s">
+      <c r="H6" s="240" t="s">
+        <v>439</v>
+      </c>
+      <c r="I6" s="241" t="s">
         <v>447</v>
       </c>
-      <c r="H6" s="240" t="s">
-        <v>440</v>
-      </c>
-      <c r="I6" s="241" t="s">
+      <c r="J6" s="241" t="s">
         <v>448</v>
       </c>
-      <c r="J6" s="241" t="s">
+      <c r="K6" s="241" t="s">
         <v>449</v>
       </c>
-      <c r="K6" s="241" t="s">
+      <c r="L6" s="241" t="s">
         <v>450</v>
       </c>
-      <c r="L6" s="241" t="s">
+      <c r="M6" s="241" t="s">
         <v>451</v>
-      </c>
-      <c r="M6" s="241" t="s">
-        <v>452</v>
       </c>
       <c r="O6" s="15" t="s">
         <v>95</v>
@@ -16886,7 +16887,7 @@
     </row>
     <row r="9" spans="2:15" x14ac:dyDescent="0.2">
       <c r="B9" s="12" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="C9" s="12" t="s">
         <v>25</v>
@@ -16930,7 +16931,7 @@
     </row>
     <row r="10" spans="2:15" x14ac:dyDescent="0.2">
       <c r="B10" s="77" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="C10" s="77" t="s">
         <v>25</v>
@@ -17246,7 +17247,7 @@
     </row>
     <row r="19" spans="2:15" x14ac:dyDescent="0.2">
       <c r="B19" s="7" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="C19" s="7" t="s">
         <v>25</v>
@@ -17436,7 +17437,7 @@
         <v>14.852708840467759</v>
       </c>
       <c r="O24" s="14" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
     </row>
     <row r="25" spans="2:15" x14ac:dyDescent="0.2">
@@ -17480,7 +17481,7 @@
         <v>560.50265585129762</v>
       </c>
       <c r="O25" s="14" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
     </row>
     <row r="26" spans="2:15" x14ac:dyDescent="0.2">
@@ -17631,7 +17632,7 @@
         <v>23.354277327137421</v>
       </c>
       <c r="O30" s="14" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
     </row>
     <row r="31" spans="2:15" x14ac:dyDescent="0.2">
@@ -17863,7 +17864,7 @@
         <v>1158.5784579528226</v>
       </c>
       <c r="O37" s="14" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
     </row>
     <row r="38" spans="1:15" x14ac:dyDescent="0.2">
@@ -18099,7 +18100,7 @@
     </row>
     <row r="45" spans="1:15" ht="15" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B45" s="5" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="C45" s="5"/>
       <c r="D45" s="5"/>
@@ -18180,34 +18181,34 @@
         <v>13</v>
       </c>
       <c r="D6" s="240" t="s">
+        <v>443</v>
+      </c>
+      <c r="E6" s="240" t="s">
         <v>444</v>
       </c>
-      <c r="E6" s="240" t="s">
+      <c r="F6" s="240" t="s">
         <v>445</v>
       </c>
-      <c r="F6" s="240" t="s">
+      <c r="G6" s="240" t="s">
         <v>446</v>
       </c>
-      <c r="G6" s="240" t="s">
+      <c r="H6" s="240" t="s">
+        <v>439</v>
+      </c>
+      <c r="I6" s="241" t="s">
         <v>447</v>
       </c>
-      <c r="H6" s="240" t="s">
-        <v>440</v>
-      </c>
-      <c r="I6" s="241" t="s">
+      <c r="J6" s="241" t="s">
         <v>448</v>
       </c>
-      <c r="J6" s="241" t="s">
+      <c r="K6" s="241" t="s">
         <v>449</v>
       </c>
-      <c r="K6" s="241" t="s">
+      <c r="L6" s="241" t="s">
         <v>450</v>
       </c>
-      <c r="L6" s="241" t="s">
+      <c r="M6" s="241" t="s">
         <v>451</v>
-      </c>
-      <c r="M6" s="241" t="s">
-        <v>452</v>
       </c>
       <c r="O6" s="15" t="s">
         <v>95</v>
@@ -18325,7 +18326,7 @@
         <v>10.704043774937976</v>
       </c>
       <c r="O10" s="5" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
     </row>
     <row r="11" spans="2:15" x14ac:dyDescent="0.2">
@@ -18376,7 +18377,7 @@
         <v>97.309488863072488</v>
       </c>
       <c r="O11" s="5" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
     </row>
     <row r="12" spans="2:15" x14ac:dyDescent="0.2">
@@ -18519,7 +18520,7 @@
         <v>-9.7309488863072495</v>
       </c>
       <c r="O14" s="1" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
     </row>
     <row r="15" spans="2:15" x14ac:dyDescent="0.2">
@@ -18728,7 +18729,7 @@
         <v>-61.067817866576291</v>
       </c>
       <c r="O20" s="1" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
     </row>
     <row r="21" spans="2:15" x14ac:dyDescent="0.2">
@@ -18845,7 +18846,7 @@
         <v>-317.91026951269441</v>
       </c>
       <c r="O24" s="5" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
     </row>
     <row r="25" spans="2:15" x14ac:dyDescent="0.2">
@@ -19186,7 +19187,7 @@
         <v>476.48007807694847</v>
       </c>
       <c r="O33" s="1" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
     </row>
     <row r="34" spans="2:15" x14ac:dyDescent="0.2">
@@ -19457,7 +19458,7 @@
         <v>15.022291609217127</v>
       </c>
       <c r="O40" s="5" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
     </row>
     <row r="41" spans="2:15" x14ac:dyDescent="0.2">

</xml_diff>